<commit_message>
Fix directed baselines and Hits@K evaluation
</commit_message>
<xml_diff>
--- a/results/link_results.xlsx
+++ b/results/link_results.xlsx
@@ -585,22 +585,22 @@
         <v>200</v>
       </c>
       <c r="I2" t="n">
-        <v>0.7886</v>
+        <v>0.7952</v>
       </c>
       <c r="J2" t="n">
-        <v>0.8027</v>
+        <v>0.805</v>
       </c>
       <c r="K2" t="n">
-        <v>0.7204</v>
+        <v>0.7295</v>
       </c>
       <c r="L2" t="n">
-        <v>0.6711</v>
+        <v>0.9</v>
       </c>
       <c r="M2" t="n">
-        <v>0.5</v>
+        <v>0.6561</v>
       </c>
       <c r="N2" t="n">
-        <v>0.5</v>
+        <v>0.6551</v>
       </c>
       <c r="O2" t="n">
         <v>0.6667</v>
@@ -609,10 +609,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.5</v>
+        <v>0.6561</v>
       </c>
       <c r="R2" t="n">
-        <v>0.5</v>
+        <v>0.6558</v>
       </c>
       <c r="S2" t="n">
         <v>0.6667</v>
@@ -621,25 +621,25 @@
         <v>1</v>
       </c>
       <c r="U2" t="n">
-        <v>0.5</v>
+        <v>0.6256</v>
       </c>
       <c r="V2" t="n">
-        <v>0.5</v>
+        <v>0.6749000000000001</v>
       </c>
       <c r="W2" t="n">
-        <v>0.6667</v>
+        <v>0.6083</v>
       </c>
       <c r="X2" t="n">
-        <v>1</v>
+        <v>0.5019</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.93</v>
+        <v>0.6</v>
       </c>
       <c r="Z2" t="n">
         <v>48064</v>
       </c>
       <c r="AA2" t="n">
-        <v>384.54</v>
+        <v>385.45</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Complete benchmarking fixes and architecture updates
</commit_message>
<xml_diff>
--- a/results/link_results.xlsx
+++ b/results/link_results.xlsx
@@ -585,10 +585,10 @@
         <v>200</v>
       </c>
       <c r="I2" t="n">
-        <v>0.7852</v>
+        <v>0.7851</v>
       </c>
       <c r="J2" t="n">
-        <v>0.7867</v>
+        <v>0.7866</v>
       </c>
       <c r="K2" t="n">
         <v>0.733</v>
@@ -606,7 +606,7 @@
         <v>0.6667</v>
       </c>
       <c r="P2" t="n">
-        <v>1</v>
+        <v>0.9953</v>
       </c>
       <c r="Q2" t="n">
         <v>0.6562</v>
@@ -618,7 +618,7 @@
         <v>0.6667</v>
       </c>
       <c r="T2" t="n">
-        <v>1</v>
+        <v>0.9905</v>
       </c>
       <c r="U2" t="n">
         <v>0.6256</v>
@@ -630,16 +630,16 @@
         <v>0.6083</v>
       </c>
       <c r="X2" t="n">
-        <v>0.5019</v>
+        <v>0.891</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.88</v>
+        <v>1.45</v>
       </c>
       <c r="Z2" t="n">
         <v>48128</v>
       </c>
       <c r="AA2" t="n">
-        <v>386.03</v>
+        <v>397.07</v>
       </c>
     </row>
     <row r="3">
@@ -674,16 +674,16 @@
         <v>200</v>
       </c>
       <c r="I3" t="n">
-        <v>0.8866000000000001</v>
+        <v>0.7657</v>
       </c>
       <c r="J3" t="n">
-        <v>0.8917</v>
+        <v>0.7496</v>
       </c>
       <c r="K3" t="n">
-        <v>0.7739</v>
+        <v>0.7185</v>
       </c>
       <c r="L3" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="M3" t="n">
         <v>0.6561</v>
@@ -695,19 +695,19 @@
         <v>0.6667</v>
       </c>
       <c r="P3" t="n">
-        <v>1</v>
+        <v>0.9953</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.6561</v>
+        <v>0.6562</v>
       </c>
       <c r="R3" t="n">
-        <v>0.6558</v>
+        <v>0.6559</v>
       </c>
       <c r="S3" t="n">
         <v>0.6667</v>
       </c>
       <c r="T3" t="n">
-        <v>1</v>
+        <v>0.9905</v>
       </c>
       <c r="U3" t="n">
         <v>0.6256</v>
@@ -719,16 +719,16 @@
         <v>0.6083</v>
       </c>
       <c r="X3" t="n">
-        <v>0.5019</v>
+        <v>0.891</v>
       </c>
       <c r="Y3" t="n">
-        <v>3.84</v>
+        <v>1.95</v>
       </c>
       <c r="Z3" t="n">
-        <v>376416</v>
+        <v>48256</v>
       </c>
       <c r="AA3" t="n">
-        <v>470.24</v>
+        <v>405.71</v>
       </c>
     </row>
     <row r="4">
@@ -763,16 +763,16 @@
         <v>200</v>
       </c>
       <c r="I4" t="n">
-        <v>0.7875</v>
+        <v>0.7931</v>
       </c>
       <c r="J4" t="n">
-        <v>0.7818000000000001</v>
+        <v>0.7788</v>
       </c>
       <c r="K4" t="n">
-        <v>0.7388</v>
+        <v>0.7519</v>
       </c>
       <c r="L4" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="M4" t="n">
         <v>0.6561</v>
@@ -784,19 +784,19 @@
         <v>0.6667</v>
       </c>
       <c r="P4" t="n">
-        <v>1</v>
+        <v>0.9953</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.6561</v>
+        <v>0.6562</v>
       </c>
       <c r="R4" t="n">
-        <v>0.6558</v>
+        <v>0.6559</v>
       </c>
       <c r="S4" t="n">
         <v>0.6667</v>
       </c>
       <c r="T4" t="n">
-        <v>1</v>
+        <v>0.9905</v>
       </c>
       <c r="U4" t="n">
         <v>0.6256</v>
@@ -808,16 +808,16 @@
         <v>0.6083</v>
       </c>
       <c r="X4" t="n">
-        <v>0.5019</v>
+        <v>0.891</v>
       </c>
       <c r="Y4" t="n">
-        <v>2.22</v>
+        <v>1.79</v>
       </c>
       <c r="Z4" t="n">
-        <v>93888</v>
+        <v>95008</v>
       </c>
       <c r="AA4" t="n">
-        <v>466.99</v>
+        <v>481.73</v>
       </c>
     </row>
     <row r="5">
@@ -852,13 +852,13 @@
         <v>200</v>
       </c>
       <c r="I5" t="n">
-        <v>0.8128</v>
+        <v>0.7814</v>
       </c>
       <c r="J5" t="n">
-        <v>0.8247</v>
+        <v>0.8025</v>
       </c>
       <c r="K5" t="n">
-        <v>0.7407</v>
+        <v>0.7226</v>
       </c>
       <c r="L5" t="n">
         <v>1</v>
@@ -873,19 +873,19 @@
         <v>0.6667</v>
       </c>
       <c r="P5" t="n">
-        <v>1</v>
+        <v>0.9953</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.6561</v>
+        <v>0.6562</v>
       </c>
       <c r="R5" t="n">
-        <v>0.6558</v>
+        <v>0.6559</v>
       </c>
       <c r="S5" t="n">
         <v>0.6667</v>
       </c>
       <c r="T5" t="n">
-        <v>1</v>
+        <v>0.9905</v>
       </c>
       <c r="U5" t="n">
         <v>0.6256</v>
@@ -897,16 +897,16 @@
         <v>0.6083</v>
       </c>
       <c r="X5" t="n">
-        <v>0.5019</v>
+        <v>0.891</v>
       </c>
       <c r="Y5" t="n">
-        <v>4.81</v>
+        <v>3.08</v>
       </c>
       <c r="Z5" t="n">
-        <v>48064</v>
+        <v>49184</v>
       </c>
       <c r="AA5" t="n">
-        <v>450.72</v>
+        <v>464.91</v>
       </c>
     </row>
     <row r="6">
@@ -941,13 +941,13 @@
         <v>200</v>
       </c>
       <c r="I6" t="n">
-        <v>0.8021</v>
+        <v>0.802</v>
       </c>
       <c r="J6" t="n">
-        <v>0.819</v>
+        <v>0.8135</v>
       </c>
       <c r="K6" t="n">
-        <v>0.7399</v>
+        <v>0.7423999999999999</v>
       </c>
       <c r="L6" t="n">
         <v>1</v>
@@ -962,19 +962,19 @@
         <v>0.6667</v>
       </c>
       <c r="P6" t="n">
-        <v>1</v>
+        <v>0.9725</v>
       </c>
       <c r="Q6" t="n">
         <v>0.6227</v>
       </c>
       <c r="R6" t="n">
-        <v>0.6216</v>
+        <v>0.622</v>
       </c>
       <c r="S6" t="n">
         <v>0.6667</v>
       </c>
       <c r="T6" t="n">
-        <v>1</v>
+        <v>0.989</v>
       </c>
       <c r="U6" t="n">
         <v>0.586</v>
@@ -986,16 +986,16 @@
         <v>0.5584</v>
       </c>
       <c r="X6" t="n">
-        <v>0.5489000000000001</v>
+        <v>0.8846000000000001</v>
       </c>
       <c r="Y6" t="n">
-        <v>1.12</v>
+        <v>0.91</v>
       </c>
       <c r="Z6" t="n">
-        <v>120704</v>
+        <v>120768</v>
       </c>
       <c r="AA6" t="n">
-        <v>415.03</v>
+        <v>429.31</v>
       </c>
     </row>
     <row r="7">
@@ -1030,13 +1030,13 @@
         <v>200</v>
       </c>
       <c r="I7" t="n">
-        <v>0.8904</v>
+        <v>0.7849</v>
       </c>
       <c r="J7" t="n">
-        <v>0.9073</v>
+        <v>0.8048</v>
       </c>
       <c r="K7" t="n">
-        <v>0.7681</v>
+        <v>0.7184</v>
       </c>
       <c r="L7" t="n">
         <v>1</v>
@@ -1051,19 +1051,19 @@
         <v>0.6667</v>
       </c>
       <c r="P7" t="n">
-        <v>1</v>
+        <v>0.9725</v>
       </c>
       <c r="Q7" t="n">
         <v>0.6227</v>
       </c>
       <c r="R7" t="n">
-        <v>0.6216</v>
+        <v>0.622</v>
       </c>
       <c r="S7" t="n">
         <v>0.6667</v>
       </c>
       <c r="T7" t="n">
-        <v>1</v>
+        <v>0.989</v>
       </c>
       <c r="U7" t="n">
         <v>0.586</v>
@@ -1075,16 +1075,16 @@
         <v>0.5584</v>
       </c>
       <c r="X7" t="n">
-        <v>0.5489000000000001</v>
+        <v>0.8846000000000001</v>
       </c>
       <c r="Y7" t="n">
-        <v>11.07</v>
+        <v>1.05</v>
       </c>
       <c r="Z7" t="n">
-        <v>957536</v>
+        <v>120896</v>
       </c>
       <c r="AA7" t="n">
-        <v>486.24</v>
+        <v>436.04</v>
       </c>
     </row>
     <row r="8">
@@ -1119,13 +1119,13 @@
         <v>200</v>
       </c>
       <c r="I8" t="n">
-        <v>0.8004</v>
+        <v>0.7574</v>
       </c>
       <c r="J8" t="n">
-        <v>0.8033</v>
+        <v>0.7369</v>
       </c>
       <c r="K8" t="n">
-        <v>0.7403999999999999</v>
+        <v>0.7203000000000001</v>
       </c>
       <c r="L8" t="n">
         <v>1</v>
@@ -1140,19 +1140,19 @@
         <v>0.6667</v>
       </c>
       <c r="P8" t="n">
-        <v>1</v>
+        <v>0.9725</v>
       </c>
       <c r="Q8" t="n">
         <v>0.6227</v>
       </c>
       <c r="R8" t="n">
-        <v>0.6216</v>
+        <v>0.622</v>
       </c>
       <c r="S8" t="n">
         <v>0.6667</v>
       </c>
       <c r="T8" t="n">
-        <v>1</v>
+        <v>0.989</v>
       </c>
       <c r="U8" t="n">
         <v>0.586</v>
@@ -1164,16 +1164,16 @@
         <v>0.5584</v>
       </c>
       <c r="X8" t="n">
-        <v>0.5489000000000001</v>
+        <v>0.8846000000000001</v>
       </c>
       <c r="Y8" t="n">
-        <v>3.26</v>
+        <v>4.43</v>
       </c>
       <c r="Z8" t="n">
-        <v>239168</v>
+        <v>240288</v>
       </c>
       <c r="AA8" t="n">
-        <v>627.21</v>
+        <v>634.96</v>
       </c>
     </row>
     <row r="9">
@@ -1208,13 +1208,13 @@
         <v>200</v>
       </c>
       <c r="I9" t="n">
-        <v>0.7983</v>
+        <v>0.716</v>
       </c>
       <c r="J9" t="n">
-        <v>0.8016</v>
+        <v>0.7149</v>
       </c>
       <c r="K9" t="n">
-        <v>0.7467</v>
+        <v>0.702</v>
       </c>
       <c r="L9" t="n">
         <v>1</v>
@@ -1229,19 +1229,19 @@
         <v>0.6667</v>
       </c>
       <c r="P9" t="n">
-        <v>1</v>
+        <v>0.9725</v>
       </c>
       <c r="Q9" t="n">
         <v>0.6227</v>
       </c>
       <c r="R9" t="n">
-        <v>0.6216</v>
+        <v>0.622</v>
       </c>
       <c r="S9" t="n">
         <v>0.6667</v>
       </c>
       <c r="T9" t="n">
-        <v>1</v>
+        <v>0.989</v>
       </c>
       <c r="U9" t="n">
         <v>0.586</v>
@@ -1253,16 +1253,16 @@
         <v>0.5584</v>
       </c>
       <c r="X9" t="n">
-        <v>0.5489000000000001</v>
+        <v>0.8846000000000001</v>
       </c>
       <c r="Y9" t="n">
-        <v>9.48</v>
+        <v>4.06</v>
       </c>
       <c r="Z9" t="n">
-        <v>120704</v>
+        <v>121824</v>
       </c>
       <c r="AA9" t="n">
-        <v>612.72</v>
+        <v>622.8</v>
       </c>
     </row>
     <row r="10">
@@ -1297,13 +1297,13 @@
         <v>200</v>
       </c>
       <c r="I10" t="n">
-        <v>0.5253</v>
+        <v>0.9287</v>
       </c>
       <c r="J10" t="n">
-        <v>0.5877</v>
+        <v>0.9351</v>
       </c>
       <c r="K10" t="n">
-        <v>0.6666</v>
+        <v>0.802</v>
       </c>
       <c r="L10" t="n">
         <v>1</v>
@@ -1318,7 +1318,7 @@
         <v>0.6667</v>
       </c>
       <c r="P10" t="n">
-        <v>1</v>
+        <v>0.9972</v>
       </c>
       <c r="Q10" t="n">
         <v>0.6191</v>
@@ -1330,7 +1330,7 @@
         <v>0.6667</v>
       </c>
       <c r="T10" t="n">
-        <v>1</v>
+        <v>0.9949</v>
       </c>
       <c r="U10" t="n">
         <v>0.7202</v>
@@ -1342,16 +1342,16 @@
         <v>0.7042</v>
       </c>
       <c r="X10" t="n">
-        <v>0.5028</v>
+        <v>0.9549</v>
       </c>
       <c r="Y10" t="n">
-        <v>1.15</v>
+        <v>3.74</v>
       </c>
       <c r="Z10" t="n">
-        <v>18208</v>
+        <v>18272</v>
       </c>
       <c r="AA10" t="n">
-        <v>494.07</v>
+        <v>516.29</v>
       </c>
     </row>
     <row r="11">
@@ -1386,13 +1386,13 @@
         <v>200</v>
       </c>
       <c r="I11" t="n">
-        <v>0.9402</v>
+        <v>0.8826000000000001</v>
       </c>
       <c r="J11" t="n">
-        <v>0.9353</v>
+        <v>0.8771</v>
       </c>
       <c r="K11" t="n">
-        <v>0.8131</v>
+        <v>0.7786999999999999</v>
       </c>
       <c r="L11" t="n">
         <v>0.9</v>
@@ -1407,7 +1407,7 @@
         <v>0.6667</v>
       </c>
       <c r="P11" t="n">
-        <v>1</v>
+        <v>0.9972</v>
       </c>
       <c r="Q11" t="n">
         <v>0.6191</v>
@@ -1419,7 +1419,7 @@
         <v>0.6667</v>
       </c>
       <c r="T11" t="n">
-        <v>1</v>
+        <v>0.9949</v>
       </c>
       <c r="U11" t="n">
         <v>0.7202</v>
@@ -1431,16 +1431,16 @@
         <v>0.7042</v>
       </c>
       <c r="X11" t="n">
-        <v>0.5028</v>
+        <v>0.9549</v>
       </c>
       <c r="Y11" t="n">
-        <v>20.64</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="Z11" t="n">
-        <v>137568</v>
+        <v>18400</v>
       </c>
       <c r="AA11" t="n">
-        <v>848.09</v>
+        <v>572.59</v>
       </c>
     </row>
     <row r="12">
@@ -1475,16 +1475,16 @@
         <v>200</v>
       </c>
       <c r="I12" t="n">
-        <v>0.8656</v>
+        <v>0.8569</v>
       </c>
       <c r="J12" t="n">
-        <v>0.8773</v>
+        <v>0.8622</v>
       </c>
       <c r="K12" t="n">
-        <v>0.7622</v>
+        <v>0.7664</v>
       </c>
       <c r="L12" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="M12" t="n">
         <v>0.619</v>
@@ -1496,7 +1496,7 @@
         <v>0.6667</v>
       </c>
       <c r="P12" t="n">
-        <v>1</v>
+        <v>0.9972</v>
       </c>
       <c r="Q12" t="n">
         <v>0.6191</v>
@@ -1508,7 +1508,7 @@
         <v>0.6667</v>
       </c>
       <c r="T12" t="n">
-        <v>1</v>
+        <v>0.9949</v>
       </c>
       <c r="U12" t="n">
         <v>0.7202</v>
@@ -1520,16 +1520,16 @@
         <v>0.7042</v>
       </c>
       <c r="X12" t="n">
-        <v>0.5028</v>
+        <v>0.9549</v>
       </c>
       <c r="Y12" t="n">
-        <v>5.5</v>
+        <v>7.19</v>
       </c>
       <c r="Z12" t="n">
-        <v>34176</v>
+        <v>35296</v>
       </c>
       <c r="AA12" t="n">
-        <v>664.5</v>
+        <v>688.35</v>
       </c>
     </row>
     <row r="13">
@@ -1564,13 +1564,13 @@
         <v>200</v>
       </c>
       <c r="I13" t="n">
-        <v>0.7297</v>
+        <v>0.7462</v>
       </c>
       <c r="J13" t="n">
-        <v>0.7559</v>
+        <v>0.8159</v>
       </c>
       <c r="K13" t="n">
-        <v>0.6508</v>
+        <v>0.662</v>
       </c>
       <c r="L13" t="n">
         <v>1</v>
@@ -1585,7 +1585,7 @@
         <v>0.6667</v>
       </c>
       <c r="P13" t="n">
-        <v>1</v>
+        <v>0.9972</v>
       </c>
       <c r="Q13" t="n">
         <v>0.6191</v>
@@ -1597,7 +1597,7 @@
         <v>0.6667</v>
       </c>
       <c r="T13" t="n">
-        <v>1</v>
+        <v>0.9949</v>
       </c>
       <c r="U13" t="n">
         <v>0.7202</v>
@@ -1609,16 +1609,16 @@
         <v>0.7042</v>
       </c>
       <c r="X13" t="n">
-        <v>0.5028</v>
+        <v>0.9549</v>
       </c>
       <c r="Y13" t="n">
-        <v>1.87</v>
+        <v>3.33</v>
       </c>
       <c r="Z13" t="n">
-        <v>18208</v>
+        <v>19328</v>
       </c>
       <c r="AA13" t="n">
-        <v>615.23</v>
+        <v>642.26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>